<commit_message>
The ED Scenario 11 workbook gates on the open caring-contact schedule, not on two closed tool epics
Step 11.7-2A's gatingIssues named #26 (TL-010 Caring Contacts) and #28 (TL-012
ED-SAFE). Both are closed: TL-010 is built and launchable, its remaining
cadence work is now #628, and TL-012 was retired in July into the generalized
follow-up tools, whose outreach attempt (TL-033) already records each call.

- gatingIssues → #628 only.
- profileBinding names the built outreach attempt and narrows the gap to what
  is actually missing: no PlanDefinition schedules the series, neither the
  caring-contact cadence nor the ED-SAFE call protocol.
- The section note and gatingIntro stop speaking in status:planned/built
  labels, which were retired with the per-tool epics; the generated heading
  becomes "Gating issues" (generator, README and docs-gates.md follow).

Outputs regenerated with build-use-case-workbook.mjs; --check is current.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/use-cases/dist/HL7_BH_USE_CASES-ED-Scenario-11.xlsx
+++ b/docs/use-cases/dist/HL7_BH_USE_CASES-ED-Scenario-11.xlsx
@@ -2971,7 +2971,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="116" customHeight="1">
+    <row r="35" ht="172" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">11.7-2A</t>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SPiER Caring Contact (built — spier-caring-contact) — TL-010 is built and launchable at /patient/workflow/caring-contact; gap — no PlanDefinition schedules the series, and the ED-SAFE telephone protocol (TL-012) it would envelope is not modelled</t>
+          <t xml:space="preserve">SPiER Caring Contact (built — spier-caring-contact) — TL-010 is built and launchable at /patient/workflow/caring-contact, and each follow-up call is recordable as a SPiER Follow-Up Outreach Attempt (built — spier-outreach-attempt, TL-033); gap — no PlanDefinition schedules the series: neither the caring-contact cadence (#628) nor the ED-SAFE telephone-call protocol it would envelope</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">

</xml_diff>